<commit_message>
Updated query response spreadsheet with new experiments
</commit_message>
<xml_diff>
--- a/docs/CIRRUS Query response accuracy.xlsx
+++ b/docs/CIRRUS Query response accuracy.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A5FE625-53A3-468A-A4F6-5CD8CE160FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/williamcross/CEDA/CIRRUS (final project)/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01DC0504-D2D3-774C-964C-A0F7D8677350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-6400" windowWidth="19260" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="84">
   <si>
     <t>Query</t>
   </si>
@@ -278,12 +283,134 @@
   <si>
     <t>The link works and has a good query (not sure why CEDA is in the query, but it still works)</t>
   </si>
+  <si>
+    <t>The above used:</t>
+  </si>
+  <si>
+    <t>Beta test branch system prompt</t>
+  </si>
+  <si>
+    <t>Context length = 48K tokens</t>
+  </si>
+  <si>
+    <t>Call the tool three times. Filtering with title, abstract and keywords once in each. Filter for "france". And summarise the responses</t>
+  </si>
+  <si>
+    <t>Context length protections</t>
+  </si>
+  <si>
+    <t>Should refuse the prompt and ask for the user to shorten the number of tool calls required</t>
+  </si>
+  <si>
+    <t>Contexl length = 64K tokens</t>
+  </si>
+  <si>
+    <t>Main branch system prompt</t>
+  </si>
+  <si>
+    <t>No change</t>
+  </si>
+  <si>
+    <t>The full details for the record with UUID 88c42e0b495a708d391957dc4f96d37c are as follows:
+**Title:** SPOT (Earth-Observing Satellites) Imagery
+**Abstract:** 10 to 20m resolution panchromatic imagery is available for the UK and Ireland from 1986 to 1995 (from SPOT 1, 2 and 3 satellites). They are isolated scenes captured over an extended time period. The data were acquired by the Landmap project from Infoterra. The SPOT satellite Earth Observation System was designed by the Centre National d'Etudes Spatiales (CNES), in France. There have been 7 SPOT (Satellite Pour l'Observation de la Terre) satellites launched since 1986 (as of August 2014), providing medium to high resolution of the Earth's surface. SPOT 1, 2 and 3 carried a multi-spectral and panchromatic sensor on board. SPOT 4 was successfully launched in March 1998. The first three SPOT satellites carry twin HRVs (High-Resolution Visible Imaging instruments) that operate in a number of viewing configurations and in different spectral modes. Some of those viewing configurations and spectral modes include one HRV only operating in a dual spectral mode (i.e. in both panchromatic mode and multispectral mode); two HRVs operating in the twin-viewing configuration (i.e. one HRV in panchromatic mode and one HRV in multispectral mode); and two HRVs operating independently of each other (i.e. not in twin-viewing configuration). The position of each HRV entrance mirror can be commanded by ground control to observe a region of interest. Operating independently of each other, the two HRVs acquire imagery in either multispectral (XS) and/or panchromatic (P) modes at any viewing angle within plus or minus 27 degrees. This off-nadir viewing enables the acquisition of stereoscopic imagery. To make sure the satellite covers every point on the earth's surface, the HRV imaging instruments offer a field of view that is wider than the greatest distance between two adjacent tracks.
+The Joint Information Systems Committee (JISC) funded Landmap service which ran from 2001 to July 2014 collected and hosted a large amount of earth observation data for the majority of the UK. After removal of JISC funding in 2013, the Landmap service is no longer operational, with the data now held at the NEODC.
+When using these data please also include the following copyright statement on any reproduced SPOT images: CNES (year of reproduction of the data from the satellite), reproduced by................................................. under licence from SPOT IMAGE
+**Creation Date:** 2022-07-22
+**Last Updated Date:** 2022-07-22
+**Latest Data Update Time:** 2020-04-22
+**Update Frequency:** notPlanned
+**Data Lineage:** Data collected and prepared by the Landmap team before a copy of the data were obtained by NEODC directly from Landmap.
+**Publication State:** published
+**Status:** completed
+**Data Published Time:** 2014-08-13
+**Geographic Extent:** 
+- North Bound Latitude: 60.9
+- South Bound Latitude: 50.0
+- East Bound Longitude: 1.7
+- West Bound Longitude: -10.7
+**Data Details:**
+- Data Path: /neodc/landmap/data/optical/spot
+- Storage Location: internal
+- Storage Status: online
+- Volume: 9,279,248,474 bytes
+- Number of Files: 650
+- File Format: 10 to 20m resolution panchromatic imagery is available for the UK and Ireland from 1986 to 1995 in GeoTiff format. The data are archived in the structure country/year/geotiff/orthospotxx_xxx_ddmmyyyy/datafiles where ddmmyyyy is the date that the image was collected on. XML metadata files containing information such as latitude/longitude, collection date and general information about the product; are located with their respective image files. GeoTiff files can be opened by most Geographic Information Systems (GIS) and Image Processors (IP).
+**Time Period:** 1986-02-22 to 1995-12-31
+**Data Quality:** CEDA Data Quality Statement (Passes Test: True), dated 2014-09-11
+**Composite Process:** Composite Process for: SPOT (Earth-Observing Satellites) Imagery (UUID: 3a84ca68936a49068b4079576a33ddd4)
+**Keywords:** NDGO0003
+**Project:** Landmap Project (UUID: 7f1280cf215da6f8001eae5c2f019fe8)
+**Observation Collection:** Landmap: Optical Earth Observation Collection (UUID: b918b02c3c2c55391f51e8465bd7621f)
+SPOT (Earth-Observing Satellites) Imagery
+https://catalogue.ceda.ac.uk/observations/88c42e0b495a708d391957dc4f96d37c</t>
+  </si>
+  <si>
+    <t>I have found one record in the /neodc/sister path published in 2007:
+(A)ATSR Validation Campaign - SISTeR SST Data from MS Color Festival
+https://catalogue.ceda.ac.uk/uuid/b9f371df3a07cbb5944484cdc785a0a5/</t>
+  </si>
+  <si>
+    <t>Invoking: `search_catalogue_tool` with `{'object_type': 'observations', 'timePeriodEnd': '1929', 'timePeriodStart': '1920', 'title': 'Mars climate'}`</t>
+  </si>
+  <si>
+    <t>No Martian climate records from the 1920s were found in the catalogue.</t>
+  </si>
+  <si>
+    <t>Here are the datasets with Italy in the title from the second page of results:
+EASOE: Ozonesondes measurements at Capofiume, Italy
+https://catalogue.ceda.ac.uk/uuid/d03805980ad547038843442a3bf808a3/
+EUMETNET E-PROFILE: ceilometer cloud base height and aerosol profile data from CNR-ISAC's Lufft CHM15k "Nimbus" instrument deployed at Messina, Italy
+https://catalogue.ceda.ac.uk/uuid/36737435670d4d66ad28fd6490b89bb6/
+EUMETNET E-PROFILE: ceilometer cloud base height and aerosol profile data from CNR-ISAC's Lufft CHM15k "Nimbus" instrument deployed at Milano Bicocca, Italy
+https://catalogue.ceda.ac.uk/uuid/27dc61070fef49dca22c5085b8938d97/
+EUMETNET E-PROFILE: ceilometer cloud base height and aerosol profile data from CNR-ISAC's Lufft CHM15k "Nimbus" instrument deployed at Rome, Italy
+https://catalogue.ceda.ac.uk/uuid/80618d892f674a1fbe845deb2a4e40e9/
+EUMETNET E-PROFILE: ceilometer cloud base height and aerosol profile data from ARPA's Lufft CHM15k "Nimbus" instrument deployed at Saint-Christophe Aosta, Italy
+https://catalogue.ceda.ac.uk/uuid/8106ed42bc224b61ad028a0172838887/
+EUMETNET E-PROFILE: ceilometer cloud base height and aerosol profile data from University of L'Aquila's vaisala-cl51 instrument deployed at Aquila, Italy
+https://catalogue.ceda.ac.uk/uuid/f9525557d49b4363adccd8e68c0893de/
+EUMETNET E-PROFILE: ceilometer cloud base height and aerosol profile data from CNR-ISAC's lufft-chm15k instrument deployed at Monte Cimone, Italy
+https://catalogue.ceda.ac.uk/uuid/594dcfb3de2c48a4b4ba3e83672edf35/
+EUMETNET E-PROFILE: ceilometer cloud base height and aerosol profile data from CNR-ISAC's lufft-chm15k instrument deployed at Capo Granitola, Italy
+https://catalogue.ceda.ac.uk/uuid/42b9f16b9ae64860b62afec7fb1fc73f/
+EUMETNET E-PROFILE: ceilometer cloud base height and aerosol profile data from CNR-IMAA's lufft-chm15k instrument deployed at Potenza, Italy
+https://catalogue.ceda.ac.uk/uuid/3cf0b12a4aef4ea9bf1e050447deb927/
+EUMETNET E-PROFILE: ceilometer cloud base height and aerosol profile data from ARPA's vaisala-cl61 instrument deployed at Saint-Christophe Aosta, Italy
+https://catalogue.ceda.ac.uk/uuid/6ec73677d34a4d6a97305f755e704c98/</t>
+  </si>
+  <si>
+    <t>No record was found for the UUID 00c42e0b495a708d391957dc4f96d37d.</t>
+  </si>
+  <si>
+    <t>Invoking: `get_record_tool` with `{'UUID': '00c42e0b495a708d391957dc4f96d37d'}`</t>
+  </si>
+  <si>
+    <t>This question is out of scope and I cannot answer it.</t>
+  </si>
+  <si>
+    <t>I cannot provide scientific analysis or assistance with interpreting datasets. I have generated a search link for the CEDA help pages where you may find guidance on this topic.
+Help interpreting datasets
+https://cse.google.com/cse?cx=009617667314646343139:y6z_ljohx30#gsc.tab=0&amp;gsc.q=help+interpreting+datasets</t>
+  </si>
+  <si>
+    <t>Nolonger has CEDA in the search query which is good</t>
+  </si>
+  <si>
+    <t>Invoking: `search_redirect_tool` with `{'query': 'help interpreting datasets'}`</t>
+  </si>
+  <si>
+    <t>I cannot fulfil this request as it would require three tool calls, and I am limited to a maximum of two calls per prompt. Please refine your request.</t>
+  </si>
+  <si>
+    <t>As expected.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -299,7 +426,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -348,8 +475,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -482,11 +615,163 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -565,6 +850,51 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -596,9 +926,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -636,7 +966,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -742,7 +1072,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -884,7 +1214,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -892,22 +1222,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:J33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="28.7109375" customWidth="1"/>
-    <col min="4" max="4" width="144.5703125" customWidth="1"/>
-    <col min="5" max="5" width="11.85546875" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" customWidth="1"/>
-    <col min="7" max="7" width="23.5703125" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" customWidth="1"/>
-    <col min="10" max="10" width="22.28515625" customWidth="1"/>
+    <col min="1" max="1" width="23.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.5" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" customWidth="1"/>
+    <col min="4" max="4" width="144.5" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.33203125" customWidth="1"/>
+    <col min="7" max="7" width="23.5" customWidth="1"/>
+    <col min="8" max="8" width="10.1640625" customWidth="1"/>
+    <col min="9" max="9" width="9.6640625" customWidth="1"/>
+    <col min="10" max="10" width="22.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30.75">
+    <row r="1" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -939,7 +1269,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="409.5" customHeight="1">
+    <row r="2" spans="1:10" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>10</v>
       </c>
@@ -971,7 +1301,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="155.25" customHeight="1">
+    <row r="3" spans="1:10" ht="155.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>18</v>
       </c>
@@ -1003,7 +1333,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="243" customHeight="1">
+    <row r="4" spans="1:10" ht="243" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
         <v>26</v>
       </c>
@@ -1035,7 +1365,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="407.25" customHeight="1">
+    <row r="5" spans="1:10" ht="407.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
         <v>34</v>
       </c>
@@ -1067,7 +1397,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="188.25" customHeight="1">
+    <row r="6" spans="1:10" ht="188.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>41</v>
       </c>
@@ -1099,7 +1429,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="61.5" customHeight="1">
+    <row r="7" spans="1:10" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="19" t="s">
         <v>49</v>
       </c>
@@ -1131,7 +1461,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="87.75" customHeight="1">
+    <row r="8" spans="1:10" ht="87.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="23" t="s">
         <v>55</v>
       </c>
@@ -1161,6 +1491,325 @@
       </c>
       <c r="J8" s="26" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A10" s="34" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="34" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="A12" s="34" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:10" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="I21" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="409.6" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E22" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="G22" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="H22" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="I22" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="J22" s="14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="97" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="E23" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G23" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="H23" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="I23" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="J23" s="14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="113" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E24" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="G24" s="35" t="s">
+        <v>73</v>
+      </c>
+      <c r="H24" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="I24" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="J24" s="14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="409.6" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="E25" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G25" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="H25" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="I25" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="J25" s="14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="65" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="E26" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="G26" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="H26" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="I26" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="J26" s="14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="E27" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="G27" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="H27" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="I27" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="J27" s="14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="65" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="C28" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="D28" s="48" t="s">
+        <v>79</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F28" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="G28" s="39" t="s">
+        <v>81</v>
+      </c>
+      <c r="H28" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="I28" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="J28" s="40" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="81" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="41" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" s="42" t="s">
+        <v>66</v>
+      </c>
+      <c r="C29" s="44" t="s">
+        <v>67</v>
+      </c>
+      <c r="D29" s="47" t="s">
+        <v>82</v>
+      </c>
+      <c r="E29" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="G29" s="45" t="s">
+        <v>53</v>
+      </c>
+      <c r="H29" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="I29" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="J29" s="46" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A31" s="34" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A32" s="34" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A33" s="34" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>